<commit_message>
Word date-validation message by temporal kind, with format
</commit_message>
<xml_diff>
--- a/src/Excelsior.Tests/DateFormats.Test.verified.xlsx
+++ b/src/Excelsior.Tests/DateFormats.Test.verified.xlsx
@@ -102,11 +102,11 @@
       <formula1>2</formula1>
       <formula2>2958465</formula2>
     </dataValidation>
-    <dataValidation type="date" operator="between" allowBlank="1" showErrorMessage="1" errorTitle="Invalid value" error="Must be a valid date." sqref="B2:B2">
+    <dataValidation type="date" operator="between" allowBlank="1" showErrorMessage="1" errorTitle="Invalid value" error="Must be a valid date and time." sqref="B2:B2">
       <formula1>2</formula1>
       <formula2>2958465</formula2>
     </dataValidation>
-    <dataValidation type="date" operator="between" allowBlank="1" showErrorMessage="1" errorTitle="Invalid value" error="Must be a valid date." sqref="C2:C2">
+    <dataValidation type="date" operator="between" allowBlank="1" showErrorMessage="1" errorTitle="Invalid value" error="Must be a valid date and time." sqref="C2:C2">
       <formula1>2</formula1>
       <formula2>2958465</formula2>
     </dataValidation>

</xml_diff>

<commit_message>
Preserve sub-hour offsets in DateTimeOffset round-trip
DefaultDateTimeOffsetFormat used `z` (whole-hour offset), so +05:30 was
written as +5 and read back as +05:00 — shifting the instant by 30/45 min
for India/Nepal-style zones. Use `zzz` to emit the full offset.
</commit_message>
<xml_diff>
--- a/src/Excelsior.Tests/DateFormats.Test.verified.xlsx
+++ b/src/Excelsior.Tests/DateFormats.Test.verified.xlsx
@@ -91,7 +91,7 @@
       </c>
       <c r="C2" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">2020-10-01 06:30:00 +11</t>
+          <t xml:space="preserve">2020-10-01 06:30:00 +11:00</t>
         </is>
       </c>
     </row>
@@ -106,7 +106,7 @@
       <formula1>2</formula1>
       <formula2>2958465</formula2>
     </dataValidation>
-    <dataValidation type="date" operator="between" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid value" error="Must be a valid date and time.&#10;yyyy-MM-dd HH:mm:ss z" prompt="Date and time as yyyy-MM-dd HH:mm:ss z" sqref="C2:C2">
+    <dataValidation type="date" operator="between" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid value" error="Must be a valid date and time.&#10;yyyy-MM-dd HH:mm:ss zzz" prompt="Date and time as yyyy-MM-dd HH:mm:ss zzz" sqref="C2:C2">
       <formula1>2</formula1>
       <formula2>2958465</formula2>
     </dataValidation>

</xml_diff>

<commit_message>
Preserve sub-hour offsets in DateTimeOffset round-trip (#239)
DefaultDateTimeOffsetFormat used `z` (whole-hour offset), so +05:30 was
written as +5 and read back as +05:00 — shifting the instant by 30/45 min
for India/Nepal-style zones. Use `zzz` to emit the full offset.
</commit_message>
<xml_diff>
--- a/src/Excelsior.Tests/DateFormats.Test.verified.xlsx
+++ b/src/Excelsior.Tests/DateFormats.Test.verified.xlsx
@@ -91,7 +91,7 @@
       </c>
       <c r="C2" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">2020-10-01 06:30:00 +11</t>
+          <t xml:space="preserve">2020-10-01 06:30:00 +11:00</t>
         </is>
       </c>
     </row>
@@ -106,7 +106,7 @@
       <formula1>2</formula1>
       <formula2>2958465</formula2>
     </dataValidation>
-    <dataValidation type="date" operator="between" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid value" error="Must be a valid date and time.&#10;yyyy-MM-dd HH:mm:ss z" prompt="Date and time as yyyy-MM-dd HH:mm:ss z" sqref="C2:C2">
+    <dataValidation type="date" operator="between" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid value" error="Must be a valid date and time.&#10;yyyy-MM-dd HH:mm:ss zzz" prompt="Date and time as yyyy-MM-dd HH:mm:ss zzz" sqref="C2:C2">
       <formula1>2</formula1>
       <formula2>2958465</formula2>
     </dataValidation>

</xml_diff>